<commit_message>
Lock Cumberland Utilization at 23% with 7 sets
8 GSF set-days (Manual/Guardian) ÷ (7×5 weekdays) = 8÷35 ≈ 23%.

Co-authored-by: echenry6f <echenry6f@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Cumberland_Aug17-23_Utilization_Estimate.xlsx
+++ b/Cumberland_Aug17-23_Utilization_Estimate.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,10 +46,22 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="36"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <i val="1"/>
+      <color rgb="00833C0C"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -64,6 +76,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -103,24 +125,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -486,789 +509,617 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GSF Utilization estimate — Cumberland · from PDF (Roads Export)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="55" customHeight="1">
+          <t>GSF Utilization — Cumberland · 17–23 Aug 2026 · 7 sets</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Reconstructed 69 job-days from column-split PDF · Dispatching=Cumberland · Dates 2026-08-17 → 2026-08-23 · W=5 weekdays · GSF Yes=10 (filt Manual/Guardian=8) · AFD mentions=20. Physical set count not stated — sensitivity table below. Unique AFDs=11 ⇒ ~6 sets if 2/set.</t>
+          <t>Source: Roads Export PDF (reconstructed) · Flagging filter: Manual Flagging / Guardian SmartFlagging only</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
+          <t>RESULT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>23%</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>8 ÷ (7 × 5) = 8 ÷ 35 = 22.86%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>FORMULA</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>In Field Sets</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>GSF Job=Yes on Manual Flagging or Guardian SmartFlagging</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Excluded</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Lane Closure GSF days (8/17, 8/18) — not in flagging filter</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Physical sets S</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>User-stated</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Weekdays W</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Mon 8/17 – Fri 8/21 (weekend excluded from capacity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Sets on Hand</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>7 × 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Utilization %</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>22.86% → 23%</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>8 ÷ 35</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>DAILY</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Dow</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Jobs</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>GSF Yes</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>GSF Yes on Manual/Guardian</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>On Hand day?</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>GSF on Manual/Guardian</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C18" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D18" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E18" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C19" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D19" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E19" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>Wed</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C20" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D20" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E20" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C21" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D21" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E21" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C22" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D22" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E22" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C23" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="D23" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="6" t="n">
+      <c r="E23" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C24" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D24" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="E24" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>GSF YES ROWS</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>GSF YES DETAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>Operator</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Counted in flagging filter?</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>In filter?</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>8/17/2026</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>Guardian SmartFlagging</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
         <is>
           <t>Bailey, Robert</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D29" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
         <is>
           <t>8/17/2026</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Lane Closure</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C30" s="13" t="inlineStr">
         <is>
           <t>Layton, Charles</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>NO — excluded</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>8/17/2026</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>Guardian SmartFlagging</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
         <is>
           <t>Manning, Aaron</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D31" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>8/18/2026</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>Guardian SmartFlagging</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>Bailey, Robert</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
         <is>
           <t>8/18/2026</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Lane Closure</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C33" s="13" t="inlineStr">
         <is>
           <t>Layton, Charles</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>NO — excluded</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>EXCLUDED</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>8/18/2026</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Manual Flagging</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Manual Flagging</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
         <is>
           <t>Manning, Aaron</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>8/19/2026</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>Guardian SmartFlagging</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C35" s="11" t="inlineStr">
         <is>
           <t>Bailey, Robert</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D35" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t>8/20/2026</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
         <is>
           <t>Guardian SmartFlagging</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
         <is>
           <t>Bailey, Robert</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D36" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t>8/20/2026</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>Guardian SmartFlagging</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C37" s="11" t="inlineStr">
         <is>
           <t>Fair, William</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D37" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
         <is>
           <t>8/21/2026</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B38" s="11" t="inlineStr">
         <is>
           <t>Guardian SmartFlagging</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C38" s="11" t="inlineStr">
         <is>
           <t>Manning, Aaron</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D38" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>UTILIZATION SENSITIVITY (S = physical sets)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>S (sets)</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>On Hand=S×5</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>Util set-days filt (8)</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>Util set-days all (10)</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>Util AFD devices (20)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B31" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>40.0%</t>
-        </is>
-      </c>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>50.0%</t>
-        </is>
-      </c>
-      <c r="E31" s="9" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="B32" s="10" t="n">
-        <v>25</v>
-      </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>32.0%</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="inlineStr">
-        <is>
-          <t>40.0%</t>
-        </is>
-      </c>
-      <c r="E32" s="10" t="inlineStr">
-        <is>
-          <t>80.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="B33" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>26.7%</t>
-        </is>
-      </c>
-      <c r="D33" s="10" t="inlineStr">
-        <is>
-          <t>33.3%</t>
-        </is>
-      </c>
-      <c r="E33" s="10" t="inlineStr">
-        <is>
-          <t>66.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B34" s="9" t="n">
-        <v>35</v>
-      </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t>22.9%</t>
-        </is>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
-        <is>
-          <t>28.6%</t>
-        </is>
-      </c>
-      <c r="E34" s="9" t="inlineStr">
-        <is>
-          <t>57.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B35" s="9" t="n">
-        <v>40</v>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>20.0%</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>25.0%</t>
-        </is>
-      </c>
-      <c r="E35" s="9" t="inlineStr">
-        <is>
-          <t>50.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B36" s="9" t="n">
-        <v>45</v>
-      </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>17.8%</t>
-        </is>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>22.2%</t>
-        </is>
-      </c>
-      <c r="E36" s="9" t="inlineStr">
-        <is>
-          <t>44.4%</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="B37" s="9" t="n">
-        <v>50</v>
-      </c>
-      <c r="C37" s="9" t="inlineStr">
-        <is>
-          <t>16.0%</t>
-        </is>
-      </c>
-      <c r="D37" s="9" t="inlineStr">
-        <is>
-          <t>20.0%</t>
-        </is>
-      </c>
-      <c r="E37" s="9" t="inlineStr">
-        <is>
-          <t>40.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="9" t="n">
-        <v>11</v>
-      </c>
-      <c r="B38" s="9" t="n">
-        <v>55</v>
-      </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>14.5%</t>
-        </is>
-      </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>18.2%</t>
-        </is>
-      </c>
-      <c r="E38" s="9" t="inlineStr">
-        <is>
-          <t>36.4%</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="B39" s="9" t="n">
-        <v>60</v>
-      </c>
-      <c r="C39" s="9" t="inlineStr">
-        <is>
-          <t>13.3%</t>
-        </is>
-      </c>
-      <c r="D39" s="9" t="inlineStr">
-        <is>
-          <t>16.7%</t>
-        </is>
-      </c>
-      <c r="E39" s="9" t="inlineStr">
-        <is>
-          <t>33.3%</t>
-        </is>
-      </c>
-    </row>
     <row r="41">
-      <c r="A41" s="11" t="inlineStr">
-        <is>
-          <t>PRIMARY (Washington-style, needs your set count)</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>In Field Sets = 8 (GSF Yes on Manual Flagging / Guardian SmartFlagging)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>On Hand = S × 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Utilization = 8 ÷ (S×5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="12" t="inlineStr">
-        <is>
-          <t>If S=5 (≈ unique AFD/2): 32.0%   |   If S=6: 26.7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Device-numerator alternative (York 45%~48% style): 20÷(S×5) → S=5: 80.0%, S=6: 66.7%</t>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Alternates (S=7): all GSF types 10÷35=28.6% · AFD devices 20÷35=57.1%</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1331,8 +1182,10 @@
           <t>Road Closure</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>5</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1357,8 +1210,10 @@
           <t>Lane Shift</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>4</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1383,8 +1238,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>1</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1409,8 +1266,10 @@
           <t>Guardian SmartFlagging</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>3</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1439,8 +1298,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>2</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1465,8 +1326,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>2</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1491,8 +1354,10 @@
           <t>Lane Closure</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>2</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1521,8 +1386,10 @@
           <t>Off-Road Work</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>4</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1547,8 +1414,10 @@
           <t>Off-Road Work</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>1</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1573,8 +1442,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>1</v>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1599,8 +1470,10 @@
           <t>Guardian SmartFlagging</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>2</v>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1629,8 +1502,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>2</v>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1655,8 +1530,10 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>6</v>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1681,8 +1558,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>6</v>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1707,8 +1586,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>2</v>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1733,8 +1614,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>5</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1759,8 +1642,10 @@
           <t>Lane Shift</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>4</v>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1785,8 +1670,10 @@
           <t>Guardian SmartFlagging</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>3</v>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1815,8 +1702,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>2</v>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1841,8 +1730,10 @@
           <t>Lane Closure</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>2</v>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1871,8 +1762,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>3</v>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1897,8 +1790,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>3</v>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1923,8 +1818,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>4</v>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1949,8 +1846,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D25" t="n">
-        <v>2</v>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1979,8 +1878,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>3</v>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -2005,8 +1906,10 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="D27" t="n">
-        <v>6</v>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -2031,8 +1934,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D28" t="n">
-        <v>6</v>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -2057,8 +1962,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>4</v>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -2083,8 +1990,10 @@
           <t>Lane Shift</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>4</v>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2109,8 +2018,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>2</v>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2135,8 +2046,10 @@
           <t>Guardian SmartFlagging</t>
         </is>
       </c>
-      <c r="D32" t="n">
-        <v>3</v>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2165,8 +2078,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>2</v>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -2191,8 +2106,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>2</v>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -2217,8 +2134,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D35" t="n">
-        <v>4</v>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -2243,8 +2162,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>2</v>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -2269,8 +2190,10 @@
           <t>Lane Closure</t>
         </is>
       </c>
-      <c r="D37" t="n">
-        <v>5</v>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -2295,8 +2218,10 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="D38" t="n">
-        <v>6</v>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -2321,8 +2246,10 @@
           <t>Lane Closure</t>
         </is>
       </c>
-      <c r="D39" t="n">
-        <v>3</v>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -2347,8 +2274,10 @@
           <t>Staging</t>
         </is>
       </c>
-      <c r="D40" t="n">
-        <v>4</v>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -2373,8 +2302,10 @@
           <t>Guardian SmartFlagging</t>
         </is>
       </c>
-      <c r="D41" t="n">
-        <v>3</v>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2403,8 +2334,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D42" t="n">
-        <v>2</v>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2429,8 +2362,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D43" t="n">
-        <v>2</v>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2455,8 +2390,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D44" t="n">
-        <v>4</v>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -2481,8 +2418,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D45" t="n">
-        <v>3</v>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2507,8 +2446,10 @@
           <t>Guardian SmartFlagging</t>
         </is>
       </c>
-      <c r="D46" t="n">
-        <v>2</v>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -2537,8 +2478,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D47" t="n">
-        <v>2</v>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2563,8 +2506,10 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="D48" t="n">
-        <v>6</v>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -2589,8 +2534,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D49" t="n">
-        <v>9</v>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -2615,8 +2562,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D50" t="n">
-        <v>4</v>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -2641,8 +2590,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D51" t="n">
-        <v>2</v>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -2667,8 +2618,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D52" t="n">
-        <v>2</v>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -2693,8 +2646,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D53" t="n">
-        <v>4</v>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -2719,8 +2674,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D54" t="n">
-        <v>5</v>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -2745,8 +2702,10 @@
           <t>Guardian SmartFlagging</t>
         </is>
       </c>
-      <c r="D55" t="n">
-        <v>2</v>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -2775,8 +2734,10 @@
           <t>Internal Labour</t>
         </is>
       </c>
-      <c r="D56" t="n">
-        <v>1</v>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -2801,8 +2762,10 @@
           <t>Internal Labour</t>
         </is>
       </c>
-      <c r="D57" t="n">
-        <v>1</v>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2827,8 +2790,10 @@
           <t>Internal Labour</t>
         </is>
       </c>
-      <c r="D58" t="n">
-        <v>1</v>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -2853,8 +2818,10 @@
           <t>Internal Labour</t>
         </is>
       </c>
-      <c r="D59" t="n">
-        <v>1</v>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -2879,8 +2846,10 @@
           <t>Internal Labour</t>
         </is>
       </c>
-      <c r="D60" t="n">
-        <v>1</v>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -2905,8 +2874,10 @@
           <t>Internal Labour</t>
         </is>
       </c>
-      <c r="D61" t="n">
-        <v>1</v>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -2931,8 +2902,10 @@
           <t>Internal Labour</t>
         </is>
       </c>
-      <c r="D62" t="n">
-        <v>1</v>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -2957,8 +2930,10 @@
           <t>Internal Labour</t>
         </is>
       </c>
-      <c r="D63" t="n">
-        <v>1</v>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -2983,8 +2958,10 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="D64" t="n">
-        <v>6</v>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -3009,8 +2986,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D65" t="n">
-        <v>6</v>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -3035,8 +3014,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D66" t="n">
-        <v>6</v>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -3061,8 +3042,10 @@
           <t>Mobile</t>
         </is>
       </c>
-      <c r="D67" t="n">
-        <v>6</v>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -3087,8 +3070,10 @@
           <t>Road Closure</t>
         </is>
       </c>
-      <c r="D68" t="n">
-        <v>5</v>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -3113,8 +3098,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D69" t="n">
-        <v>5</v>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -3139,8 +3126,10 @@
           <t>Manual Flagging</t>
         </is>
       </c>
-      <c r="D70" t="n">
-        <v>6</v>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Count all GSF job-days for Cumberland (no job-type exclusions)
Include Lane Closure and any other GSF Yes rows. In Field=10,
On Hand=7×5=35 → Utilization ≈ 29%.

Co-authored-by: echenry6f <echenry6f@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Cumberland_Aug17-23_Utilization_Estimate.xlsx
+++ b/Cumberland_Aug17-23_Utilization_Estimate.xlsx
@@ -61,7 +61,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -93,11 +93,6 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F4B183"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -125,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -143,7 +138,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -509,14 +503,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -529,7 +522,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: Roads Export PDF (reconstructed) · Flagging filter: Manual Flagging / Guardian SmartFlagging only</t>
+          <t>Rule update: do NOT exclude any job codes that have GSF. In Field Sets = COUNT of all job-days with GSF Job=Yes (any Job Type).</t>
         </is>
       </c>
     </row>
@@ -543,12 +536,12 @@
     <row r="5" ht="52" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>23%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>8 ÷ (7 × 5) = 8 ÷ 35 = 22.86%</t>
+          <t>10 ÷ (7 × 5) = 10 ÷ 35 = 28.57%</t>
         </is>
       </c>
     </row>
@@ -584,143 +577,139 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>GSF Job=Yes on Manual Flagging or Guardian SmartFlagging</t>
+          <t>ALL GSF Job=Yes job-days — any Job Type (incl. Lane Closure)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Excluded</t>
+          <t>Physical sets S</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Lane Closure GSF days (8/17, 8/18) — not in flagging filter</t>
+          <t>User-stated</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Physical sets S</t>
+          <t>Weekdays W</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>User-stated</t>
+          <t>Mon 8/17 – Fri 8/21</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Weekdays W</t>
+          <t>Sets on Hand</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>35</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Mon 8/17 – Fri 8/21 (weekend excluded from capacity)</t>
+          <t>7 × 5</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Sets on Hand</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>35</t>
+          <t>Utilization %</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>28.57% → 29%</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>7 × 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Utilization %</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>22.86% → 23%</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>8 ÷ 35</t>
+          <t>10 ÷ 35</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>DAILY</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>DAILY</t>
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Dow</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Jobs</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>GSF Yes (all job types)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Dow</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>Jobs</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>GSF Yes</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>GSF on Manual/Guardian</t>
-        </is>
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Mon</t>
+          <t>Tue</t>
         </is>
       </c>
       <c r="C18" s="11" t="n">
@@ -729,103 +718,88 @@
       <c r="D18" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="E18" s="11" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Tue</t>
+          <t>Wed</t>
         </is>
       </c>
       <c r="C19" s="11" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D19" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="E19" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Wed</t>
+          <t>Thu</t>
         </is>
       </c>
       <c r="C20" s="11" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D20" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Thu</t>
+          <t>Fri</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E21" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>Fri</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="n">
-        <v>16</v>
-      </c>
-      <c r="D22" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="11" t="n">
-        <v>1</v>
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Sat</t>
+          <t>Sun</t>
         </is>
       </c>
       <c r="C23" s="12" t="n">
@@ -834,57 +808,45 @@
       <c r="D23" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="E23" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
-      <c r="B24" s="12" t="inlineStr">
-        <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C24" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D24" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="12" t="n">
-        <v>0</v>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>ALL GSF YES ROWS (none excluded)</t>
+        </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>GSF YES DETAIL</t>
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Job Type</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Operator</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>Job Type</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>Operator</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>In filter?</t>
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>8/17/2026</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Guardian SmartFlagging</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>Bailey, Robert</t>
         </is>
       </c>
     </row>
@@ -896,46 +858,36 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
+          <t>Lane Closure</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>Layton, Charles</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>8/17/2026</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
           <t>Guardian SmartFlagging</t>
         </is>
       </c>
-      <c r="C29" s="11" t="inlineStr">
-        <is>
-          <t>Bailey, Robert</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="13" t="inlineStr">
-        <is>
-          <t>8/17/2026</t>
-        </is>
-      </c>
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>Lane Closure</t>
-        </is>
-      </c>
-      <c r="C30" s="13" t="inlineStr">
-        <is>
-          <t>Layton, Charles</t>
-        </is>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
-        <is>
-          <t>EXCLUDED</t>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>Manning, Aaron</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>8/17/2026</t>
+          <t>8/18/2026</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
@@ -945,12 +897,7 @@
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>Manning, Aaron</t>
-        </is>
-      </c>
-      <c r="D31" s="11" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Bailey, Robert</t>
         </is>
       </c>
     </row>
@@ -962,68 +909,53 @@
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Guardian SmartFlagging</t>
+          <t>Lane Closure</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Bailey, Robert</t>
-        </is>
-      </c>
-      <c r="D32" s="11" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Layton, Charles</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>8/18/2026</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>Lane Closure</t>
-        </is>
-      </c>
-      <c r="C33" s="13" t="inlineStr">
-        <is>
-          <t>Layton, Charles</t>
-        </is>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
-        <is>
-          <t>EXCLUDED</t>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Manual Flagging</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>Manning, Aaron</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>8/18/2026</t>
+          <t>8/19/2026</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>Manual Flagging</t>
+          <t>Guardian SmartFlagging</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Manning, Aaron</t>
-        </is>
-      </c>
-      <c r="D34" s="11" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Bailey, Robert</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>8/19/2026</t>
+          <t>8/20/2026</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
@@ -1034,11 +966,6 @@
       <c r="C35" s="11" t="inlineStr">
         <is>
           <t>Bailey, Robert</t>
-        </is>
-      </c>
-      <c r="D35" s="11" t="inlineStr">
-        <is>
-          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1055,19 +982,14 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Bailey, Robert</t>
-        </is>
-      </c>
-      <c r="D36" s="11" t="inlineStr">
-        <is>
-          <t>YES</t>
+          <t>Fair, William</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>8/20/2026</t>
+          <t>8/21/2026</t>
         </is>
       </c>
       <c r="B37" s="11" t="inlineStr">
@@ -1077,46 +999,20 @@
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Fair, William</t>
-        </is>
-      </c>
-      <c r="D37" s="11" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="11" t="inlineStr">
-        <is>
-          <t>8/21/2026</t>
-        </is>
-      </c>
-      <c r="B38" s="11" t="inlineStr">
-        <is>
-          <t>Guardian SmartFlagging</t>
-        </is>
-      </c>
-      <c r="C38" s="11" t="inlineStr">
-        <is>
           <t>Manning, Aaron</t>
         </is>
       </c>
-      <c r="D38" s="11" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Alternates (S=7): all GSF types 10÷35=28.6% · AFD devices 20÷35=57.1%</t>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Prior (with Manual/Guardian-only filter) was 8÷35=23%. Including Lane Closure GSF days raises In Field to 10.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="A2:E2"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:B5"/>

</xml_diff>